<commit_message>
Remove daily sales and theme columns
</commit_message>
<xml_diff>
--- a/templates/选品表格-模板.xlsx
+++ b/templates/选品表格-模板.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="8">
   <si>
     <t>上架时间</t>
   </si>
@@ -19,16 +19,10 @@
     <t>参考样品图</t>
   </si>
   <si>
-    <t>日销</t>
-  </si>
-  <si>
     <t>月销</t>
   </si>
   <si>
     <t>售价</t>
-  </si>
-  <si>
-    <t>主题</t>
   </si>
   <si>
     <t>标题</t>
@@ -433,11 +427,10 @@
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="57.14285714285715" customWidth="1"/>
-    <col min="3" max="5" width="13" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="56" customWidth="1"/>
-    <col min="8" max="8" width="24" customWidth="1"/>
-    <col min="9" max="32" width="57.14285714285715" customWidth="1"/>
+    <col min="3" max="4" width="13" customWidth="1"/>
+    <col min="5" max="5" width="56" customWidth="1"/>
+    <col min="6" max="6" width="24" customWidth="1"/>
+    <col min="7" max="32" width="57.14285714285715" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="68.25" customHeight="1" spans="1:32" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -466,80 +459,80 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AF1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I1"/>
+  <autoFilter ref="A1:G1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>